<commit_message>
Remove sheet-protection password across all 8 templates
A customer reported that in real Desktop Excel (Windows), several
sheets prompted for a password when editing cells that the file
itself marks as unlocked (verified at the raw XML level: the cell
style did have protection locked="false"). Root cause unconfirmed,
but the friction is real and affects every template in the line since
they all share the same protection helper.

Fix: sheets stay protected by default (still guards formulas against
accidental edits), but no password is set anymore, so "Review >
Unprotect Sheet" now works with a single click in any app, regardless
of what triggered the original issue. Updated the in-sheet
Instrucciones text and README/pack LEEME.md files accordingly, and
regenerated + re-verified (recalc.py, 0 errors) all 8 product files
plus both bundle ZIPs.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NrmspLoz6htm8DfszsUfy1
</commit_message>
<xml_diff>
--- a/productos/01-control-gastos-personales/Control-de-Gastos-Personales.xlsx
+++ b/productos/01-control-gastos-personales/Control-de-Gastos-Personales.xlsx
@@ -123,7 +123,7 @@
     <t xml:space="preserve">7. Celdas protegidas</t>
   </si>
   <si>
-    <t xml:space="preserve">Las hojas están protegidas para que no borres fórmulas por accidente. Solo puedes escribir en las celdas resaltadas en color crema / texto azul. Si necesitas desproteger una hoja, la contraseña es: plantilla2026.</t>
+    <t xml:space="preserve">Las hojas están protegidas para que no borres fórmulas por accidente. Solo puedes escribir en las celdas resaltadas en color crema / texto azul. Si necesitas editar otra celda, ve a Revisar → Desproteger hoja (no pide contraseña).</t>
   </si>
   <si>
     <t xml:space="preserve">8. Agregar más filas</t>
@@ -1854,11 +1854,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="65243127"/>
-        <c:axId val="58090017"/>
+        <c:axId val="47238555"/>
+        <c:axId val="41613821"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="65243127"/>
+        <c:axId val="47238555"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1890,7 +1890,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="58090017"/>
+        <c:crossAx val="41613821"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1898,7 +1898,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="58090017"/>
+        <c:axId val="41613821"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1940,7 +1940,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="65243127"/>
+        <c:crossAx val="47238555"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2188,11 +2188,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="759949"/>
-        <c:axId val="40639631"/>
+        <c:axId val="79805664"/>
+        <c:axId val="40713529"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="759949"/>
+        <c:axId val="79805664"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2224,7 +2224,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="40639631"/>
+        <c:crossAx val="40713529"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2232,7 +2232,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="40639631"/>
+        <c:axId val="40713529"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2274,7 +2274,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="759949"/>
+        <c:crossAx val="79805664"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2776,7 +2776,7 @@
       <c r="F24" s="7"/>
     </row>
   </sheetData>
-  <sheetProtection sheet="true" password="ee36" formatCells="false" formatColumns="false" formatRows="false" insertRows="false" selectLockedCells="true" selectUnlockedCells="true"/>
+  <sheetProtection sheet="true" formatCells="false" formatColumns="false" formatRows="false" insertRows="false" selectLockedCells="true" selectUnlockedCells="true"/>
   <mergeCells count="16">
     <mergeCell ref="B2:F2"/>
     <mergeCell ref="B4:F6"/>
@@ -2927,7 +2927,7 @@
       <c r="C28" s="7"/>
     </row>
   </sheetData>
-  <sheetProtection sheet="true" password="ee36" formatCells="false" formatColumns="false" formatRows="false" insertRows="false" selectLockedCells="true" selectUnlockedCells="true"/>
+  <sheetProtection sheet="true" formatCells="false" formatColumns="false" formatRows="false" insertRows="false" selectLockedCells="true" selectUnlockedCells="true"/>
   <mergeCells count="18">
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="B4:C4"/>
@@ -3085,7 +3085,7 @@
       <c r="D15" s="19"/>
     </row>
   </sheetData>
-  <sheetProtection sheet="true" password="ee36" formatCells="false" formatColumns="false" formatRows="false" insertRows="false" selectLockedCells="true" selectUnlockedCells="true"/>
+  <sheetProtection sheet="true" formatCells="false" formatColumns="false" formatRows="false" insertRows="false" selectLockedCells="true" selectUnlockedCells="true"/>
   <mergeCells count="2">
     <mergeCell ref="B2:D2"/>
     <mergeCell ref="B15:D15"/>
@@ -3260,7 +3260,7 @@
       <c r="B28" s="21"/>
     </row>
   </sheetData>
-  <sheetProtection sheet="true" password="ee36" formatCells="false" formatColumns="false" formatRows="false" insertRows="false" selectLockedCells="true" selectUnlockedCells="true"/>
+  <sheetProtection sheet="true" formatCells="false" formatColumns="false" formatRows="false" insertRows="false" selectLockedCells="true" selectUnlockedCells="true"/>
   <mergeCells count="2">
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="B20:C20"/>
@@ -5930,7 +5930,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection sheet="true" password="ee36" formatCells="false" formatColumns="false" formatRows="false" insertRows="false" selectLockedCells="true" selectUnlockedCells="true"/>
+  <sheetProtection sheet="true" formatCells="false" formatColumns="false" formatRows="false" insertRows="false" selectLockedCells="true" selectUnlockedCells="true"/>
   <mergeCells count="2">
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A3:G3"/>
@@ -6565,7 +6565,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection sheet="true" password="ee36" formatCells="false" formatColumns="false" formatRows="false" insertRows="false" selectLockedCells="true" selectUnlockedCells="true"/>
+  <sheetProtection sheet="true" formatCells="false" formatColumns="false" formatRows="false" insertRows="false" selectLockedCells="true" selectUnlockedCells="true"/>
   <mergeCells count="4">
     <mergeCell ref="B2:F2"/>
     <mergeCell ref="B3:F3"/>
@@ -6669,7 +6669,7 @@
       <c r="I7" s="41"/>
     </row>
   </sheetData>
-  <sheetProtection sheet="true" password="ee36" formatCells="false" formatColumns="false" formatRows="false" insertRows="false" selectLockedCells="true" selectUnlockedCells="true"/>
+  <sheetProtection sheet="true" formatCells="false" formatColumns="false" formatRows="false" insertRows="false" selectLockedCells="true" selectUnlockedCells="true"/>
   <mergeCells count="10">
     <mergeCell ref="B2:H2"/>
     <mergeCell ref="B3:H3"/>

</xml_diff>